<commit_message>
Modalità di ricerca: alternativa stessa marca o concorrente equivalente
- Nuovo parametro 'modalita' (sito: scelta nel passo Somiglianza; Excel: riga Modalità)
- Fascia comune a tutte le marche (base/entry/media/premium/top) per confrontare marche diverse
- Tabelle serie per TCL, Philips, Sony, Panasonic: tecnologia e famiglia non dipendono più
  dalle parole del titolo (stesso TV ora combacia tra Amazon e retailer)
- Concorrente: marca diversa, stessa tecnologia, fascia ±1 penalizzata, ricerche per marca
- Le ricerche salvate con 'stessa marca' spenta diventano modalità concorrente

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01131o6sWy3pYyUj8LJptoof
</commit_message>
<xml_diff>
--- a/input_tv_matcher.xlsx
+++ b/input_tv_matcher.xlsx
@@ -1222,7 +1222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1249,53 +1249,75 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Anno target</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>2026</v>
+          <t>Modalità</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>STESSA MARCA</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Solo modelli di quest'anno</t>
+          <t>STESSA MARCA = alternativa della stessa marca (codice diverso) · CONCORRENTE = modello equivalente di un'altra marca</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Accetta anno non determinabile</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
+          <t>Anno target</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2026</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SI = accetta modelli il cui anno non si ricava dal codice/titolo (segnalati nel foglio Dettaglio)</t>
+          <t>Solo modelli di quest'anno</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Accetta anno non determinabile</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>SI = accetta modelli il cui anno non si ricava dal codice/titolo (segnalati nel foglio Dettaglio)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>Verifica pagina prodotto</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
         <is>
           <t>SI = apre ogni URL scelto per controllare che sia attivo</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"STESSA MARCA,CONCORRENTE"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>